<commit_message>
Add backup and image files to the project repository
Adds backup spreadsheet and image file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 491a60ed-3b54-48e1-858f-6a37be45fc02
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/pNtS803
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-31.xlsx
+++ b/backups/proposal-log-2026-03-31.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="60">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -53,6 +53,144 @@
   </si>
   <si>
     <t>BC Link</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Flying Pickle - Idaho Falls</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>Jake Marrujo</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>26-0188</t>
+  </si>
+  <si>
+    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
+  </si>
+  <si>
+    <t>LAX</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>Gabriel Frota</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
+  </si>
+  <si>
+    <t>26-0189</t>
+  </si>
+  <si>
+    <t>Illumina Project SOL</t>
+  </si>
+  <si>
+    <t>SAN</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>Vahid Balali</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
+  </si>
+  <si>
+    <t>26-0190</t>
+  </si>
+  <si>
+    <t>Inglewood Transit Connector RFQ</t>
+  </si>
+  <si>
+    <t>Public Facility</t>
+  </si>
+  <si>
+    <t>2026-03-25</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>Nilda Puno</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
+  </si>
+  <si>
+    <t>26-0191</t>
+  </si>
+  <si>
+    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
+  </si>
+  <si>
+    <t>PDX</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Mark Socks</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
+  </si>
+  <si>
+    <t>26-0192</t>
+  </si>
+  <si>
+    <t>UWMC ML TRU Pathology Lab</t>
+  </si>
+  <si>
+    <t>SEA</t>
+  </si>
+  <si>
+    <t>2026-03-26</t>
+  </si>
+  <si>
+    <t>Nick Jennings</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c161e5eb28c8b750d054bc</t>
+  </si>
+  <si>
+    <t>26-0193</t>
+  </si>
+  <si>
+    <t>FINN Partners at First &amp; Main</t>
+  </si>
+  <si>
+    <t>Hospitality</t>
+  </si>
+  <si>
+    <t>2026-03-19</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>Jessica Howell</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69bc538e7aaadb003896155f</t>
   </si>
 </sst>
 </file>
@@ -451,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -511,8 +649,316 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" t="s">
+        <v>14</v>
+      </c>
+      <c r="N3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" t="s">
+        <v>14</v>
+      </c>
+      <c r="N6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" t="s">
+        <v>14</v>
+      </c>
+      <c r="L7" t="s">
+        <v>14</v>
+      </c>
+      <c r="M7" t="s">
+        <v>14</v>
+      </c>
+      <c r="N7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N8" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:N8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve proposal management by adding market detection and region mapping
Update logic to correctly map GC office locations to regions and improve primary market detection for new proposals.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 7dd8ec34-7f2e-46a1-92d3-baa5a918288e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/ee7umwk
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-31.xlsx
+++ b/backups/proposal-log-2026-03-31.xlsx
@@ -70,28 +70,28 @@
     <t>Jake Marrujo</t>
   </si>
   <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>26-0188</t>
+  </si>
+  <si>
+    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
+  </si>
+  <si>
+    <t>LAX</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>Gabriel Frota</t>
+  </si>
+  <si>
     <t>Draft</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
-  </si>
-  <si>
-    <t>26-0188</t>
-  </si>
-  <si>
-    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
-  </si>
-  <si>
-    <t>LAX</t>
-  </si>
-  <si>
-    <t>2026-03-27</t>
-  </si>
-  <si>
-    <t>2026-03-24</t>
-  </si>
-  <si>
-    <t>Gabriel Frota</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
@@ -678,51 +678,51 @@
         <v>14</v>
       </c>
       <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" t="s">
         <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" t="s">
-        <v>14</v>
-      </c>
-      <c r="N2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
         <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" t="s">
-        <v>19</v>
       </c>
       <c r="K3" t="s">
         <v>14</v>
@@ -751,7 +751,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F4" t="s">
         <v>31</v>
@@ -766,7 +766,7 @@
         <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K4" t="s">
         <v>14</v>
@@ -789,7 +789,7 @@
         <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
         <v>36</v>
@@ -810,7 +810,7 @@
         <v>14</v>
       </c>
       <c r="J5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K5" t="s">
         <v>14</v>
@@ -839,7 +839,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s">
         <v>44</v>
@@ -854,7 +854,7 @@
         <v>14</v>
       </c>
       <c r="J6" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K6" t="s">
         <v>14</v>
@@ -898,7 +898,7 @@
         <v>14</v>
       </c>
       <c r="J7" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K7" t="s">
         <v>14</v>
@@ -942,7 +942,7 @@
         <v>14</v>
       </c>
       <c r="J8" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K8" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
Add estimated start and finish dates to project proposals
Update bcSync.ts to include 'expectedStart' and 'expectedFinish' fields from BuildingConnected opportunities, mapping them to 'anticipatedStart' and 'anticipatedFinish' in the proposal log entries.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8d1e7a75-6397-4ee9-ab28-807ac76c7e1a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/jQAJg02
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-31.xlsx
+++ b/backups/proposal-log-2026-03-31.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="64">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -53,6 +53,156 @@
   </si>
   <si>
     <t>BC Link</t>
+  </si>
+  <si>
+    <t>26-0200</t>
+  </si>
+  <si>
+    <t>Flying Pickle Idaho Falls</t>
+  </si>
+  <si>
+    <t>SEA</t>
+  </si>
+  <si>
+    <t>Special Projects</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Jake Marrujo</t>
+  </si>
+  <si>
+    <t>Estimating</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>26-0199</t>
+  </si>
+  <si>
+    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
+  </si>
+  <si>
+    <t>LAX</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>Gabriel Frota</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
+  </si>
+  <si>
+    <t>26-0198</t>
+  </si>
+  <si>
+    <t>Illumina Project SOL</t>
+  </si>
+  <si>
+    <t>SAN</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>Vahid Balali</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
+  </si>
+  <si>
+    <t>26-0197</t>
+  </si>
+  <si>
+    <t>Inglewood Transit Connector RFQ</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>2026-03-25</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>Nilda Puno</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
+  </si>
+  <si>
+    <t>26-0196</t>
+  </si>
+  <si>
+    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
+  </si>
+  <si>
+    <t>PDX</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Mark Socks</t>
+  </si>
+  <si>
+    <t>Lost - Note Why in Comments</t>
+  </si>
+  <si>
+    <t>NO BID - No Scope</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
+  </si>
+  <si>
+    <t>26-0195</t>
+  </si>
+  <si>
+    <t>UWMC ML TRU Pathology Lab</t>
+  </si>
+  <si>
+    <t>2026-03-26</t>
+  </si>
+  <si>
+    <t>Nick Jennings</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c161e5eb28c8b750d054bc</t>
+  </si>
+  <si>
+    <t>26-0194</t>
+  </si>
+  <si>
+    <t>FINN Partners at First &amp; Main</t>
+  </si>
+  <si>
+    <t>Hospitality</t>
+  </si>
+  <si>
+    <t>2026-03-19</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>Jessica Howell</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69bc538e7aaadb003896155f</t>
   </si>
 </sst>
 </file>
@@ -451,7 +601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -511,8 +661,316 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
+      </c>
+      <c r="N3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s">
+        <v>20</v>
+      </c>
+      <c r="M4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" t="s">
+        <v>20</v>
+      </c>
+      <c r="N7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" t="s">
+        <v>20</v>
+      </c>
+      <c r="L8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" t="s">
+        <v>20</v>
+      </c>
+      <c r="N8" t="s">
+        <v>63</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:N8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update proposal log features and rename project log to change log
Refactors the application to consolidate proposal management features into the 'Proposal Log' tool, including enhanced NBS scopes and notes functionalities, and a new status dropdown with conditional modals. The 'Project Log' has been renamed to 'Change Log' across the UI, file exports, and documentation.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d343da50-f7fd-4dcd-8a8b-c8460f0a56c7
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/B7EZaNf
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-31.xlsx
+++ b/backups/proposal-log-2026-03-31.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="66">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -101,6 +101,12 @@
   </si>
   <si>
     <t>Gabriel Frota</t>
+  </si>
+  <si>
+    <t>No Bid</t>
+  </si>
+  <si>
+    <t>Automated test note</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
@@ -734,7 +740,7 @@
         <v>20</v>
       </c>
       <c r="J3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="K3" t="s">
         <v>20</v>
@@ -743,21 +749,21 @@
         <v>20</v>
       </c>
       <c r="M3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="N3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
         <v>17</v>
@@ -766,13 +772,13 @@
         <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
       </c>
       <c r="H4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I4" t="s">
         <v>20</v>
@@ -790,33 +796,33 @@
         <v>20</v>
       </c>
       <c r="N4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I5" t="s">
         <v>20</v>
@@ -834,18 +840,18 @@
         <v>20</v>
       </c>
       <c r="N5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
@@ -854,19 +860,19 @@
         <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
       </c>
       <c r="H6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I6" t="s">
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
         <v>20</v>
@@ -875,18 +881,18 @@
         <v>20</v>
       </c>
       <c r="M6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="N6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
         <v>16</v>
@@ -895,16 +901,16 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I7" t="s">
         <v>20</v>
@@ -922,33 +928,33 @@
         <v>20</v>
       </c>
       <c r="N7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
         <v>20</v>
@@ -966,7 +972,7 @@
         <v>20</v>
       </c>
       <c r="N8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>